<commit_message>
push the form part
</commit_message>
<xml_diff>
--- a/multipleupload.xlsx
+++ b/multipleupload.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>FULLNAME</t>
   </si>
@@ -32,39 +32,18 @@
     <t>EMAIL</t>
   </si>
   <si>
-    <t>SEX</t>
-  </si>
-  <si>
     <t>PHONENUMBER</t>
   </si>
   <si>
     <t>ADDRESS</t>
   </si>
   <si>
-    <t>ola kunle</t>
-  </si>
-  <si>
-    <t>b@gmail.com</t>
-  </si>
-  <si>
     <t>MALE</t>
   </si>
   <si>
-    <t>kogi</t>
-  </si>
-  <si>
-    <t>mos ini</t>
-  </si>
-  <si>
-    <t>c@gmail.com</t>
-  </si>
-  <si>
     <t>FEMALE</t>
   </si>
   <si>
-    <t>lagos</t>
-  </si>
-  <si>
     <t>olubiyomercy@gmail.com</t>
   </si>
   <si>
@@ -105,24 +84,19 @@
   </si>
   <si>
     <t>Promise Agba</t>
+  </si>
+  <si>
+    <t>GENDER</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -145,16 +119,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -433,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.6640625" customWidth="1"/>
@@ -451,152 +422,114 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
       <c r="D2">
-        <v>9876543212</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>9876543210</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D4">
-        <v>213</v>
+        <v>4321</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5">
-        <v>123</v>
+        <v>43112</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D6">
-        <v>4321</v>
+        <v>6421</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D7">
-        <v>43112</v>
+        <v>987654</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D8">
-        <v>6421</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9">
-        <v>987654</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10">
         <v>643</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
-    <hyperlink ref="B3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>